<commit_message>
implatação do modulo de cota aprendiz
</commit_message>
<xml_diff>
--- a/assets/modelos_importacao/modelo_importacao_cbo.xlsx
+++ b/assets/modelos_importacao/modelo_importacao_cbo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alcidesdiogenes\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alcidesdiogenes\Desktop\Projetos\ferramentas-dp\assets\modelos_importacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0134D9B-0001-4B83-A79A-3D6789F6C88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2429C7F-62E4-40FD-961F-F918A048E488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{42632266-C8D1-4E99-8617-BC70E36B0764}"/>
+    <workbookView xWindow="-21720" yWindow="1305" windowWidth="21840" windowHeight="13020" xr2:uid="{42632266-C8D1-4E99-8617-BC70E36B0764}"/>
   </bookViews>
   <sheets>
     <sheet name="cbo_escolaridade_estruturado" sheetId="1" r:id="rId1"/>

</xml_diff>